<commit_message>
Actualizar codigo y agregar nuevas interfaces y tests
</commit_message>
<xml_diff>
--- a/specification_generator/PROYECTOIA/METODOS_LAB/METODOS_LAB_UNIFICADO.xlsx
+++ b/specification_generator/PROYECTOIA/METODOS_LAB/METODOS_LAB_UNIFICADO.xlsx
@@ -521,12 +521,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -617,12 +617,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -713,12 +713,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -873,12 +873,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -905,12 +905,12 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1129,12 +1129,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1257,12 +1257,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -1865,12 +1865,12 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -1897,12 +1897,12 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -1961,12 +1961,12 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -1993,12 +1993,12 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -2089,12 +2089,12 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
@@ -2121,12 +2121,12 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
@@ -2153,12 +2153,12 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
@@ -2185,12 +2185,12 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -2217,12 +2217,12 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
@@ -2249,12 +2249,12 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -2281,12 +2281,12 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -2313,12 +2313,12 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
@@ -2345,12 +2345,12 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
@@ -2409,12 +2409,12 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
@@ -2441,12 +2441,12 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -2473,12 +2473,12 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
@@ -2505,12 +2505,12 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
@@ -2537,12 +2537,12 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
@@ -2569,12 +2569,12 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
@@ -2601,12 +2601,12 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
@@ -2665,12 +2665,12 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
@@ -2697,12 +2697,12 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
@@ -2729,12 +2729,12 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
@@ -2761,12 +2761,12 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
@@ -2825,12 +2825,12 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
@@ -2889,12 +2889,12 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
@@ -3017,12 +3017,12 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
@@ -3049,12 +3049,12 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
@@ -3081,12 +3081,12 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
@@ -3113,12 +3113,12 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
@@ -3145,12 +3145,12 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
@@ -3205,12 +3205,12 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
@@ -3269,12 +3269,12 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
@@ -4165,12 +4165,12 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F116" s="3" t="inlineStr">
@@ -4501,12 +4501,12 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
@@ -4529,12 +4529,12 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F129" s="3" t="inlineStr">
@@ -6293,12 +6293,12 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F192" s="3" t="inlineStr">
@@ -6349,12 +6349,12 @@
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F194" s="3" t="inlineStr">
@@ -6412,7 +6412,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-09T14:23:35</t>
+          <t>2026-10-11T22:19:32</t>
         </is>
       </c>
     </row>

</xml_diff>